<commit_message>
feature/advance/forgot password -> verify otp using java email seeder
</commit_message>
<xml_diff>
--- a/docs/Calendar.xlsx
+++ b/docs/Calendar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\fullstack\Personal Finance Management\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FCE1E6C-B3A8-4846-893C-0736C371F343}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3687F7C-7FC2-4D34-A26C-00C8F5E4B7BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -73,7 +73,7 @@
     <t>Phát triển chức năng nâng cao: Tích hợp AI, kiểm thử lần cuối</t>
   </si>
   <si>
-    <t>Hoàn thiện chức năng nâng cao: Liên kết đăng nhập (OAuth2), email xác thực (Java email seeder), ghi nhớ đăng nhập, revoke token (Redis)</t>
+    <t>Hoàn thiện chức năng nâng cao: Liên kết đăng nhập (OAuth2), email xác thực (Java email seeder), ghi nhớ đăng nhập, revoke token (Redis), lưu ảnh hồ sơ (cloudinary)</t>
   </si>
 </sst>
 </file>
@@ -137,10 +137,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -423,69 +423,69 @@
       <c r="I3" s="2"/>
     </row>
     <row r="4" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="7"/>
+      <c r="G4" s="6"/>
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
     </row>
     <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="7"/>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
+      <c r="A5" s="6"/>
+      <c r="B5" s="6"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
     </row>
     <row r="6" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="7"/>
-      <c r="B6" s="7"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
+      <c r="A6" s="6"/>
+      <c r="B6" s="6"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
     </row>
     <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="7"/>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
+      <c r="A7" s="6"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
     </row>
     <row r="8" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="7"/>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
+      <c r="A8" s="6"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="6"/>
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
     </row>
@@ -515,65 +515,65 @@
       <c r="I9" s="2"/>
     </row>
     <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7" t="s">
+      <c r="C10" s="6"/>
+      <c r="D10" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
     </row>
     <row r="11" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="7"/>
-      <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
+      <c r="A11" s="6"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
     </row>
     <row r="12" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="7"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
       <c r="H12" s="3"/>
       <c r="I12" s="3"/>
     </row>
     <row r="13" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="7"/>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
+      <c r="A13" s="6"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
     </row>
     <row r="14" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="7"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
+      <c r="A14" s="6"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
     </row>

</xml_diff>

<commit_message>
[v2: done] Last updated search, category classification [using Gemini], UI, and system language
</commit_message>
<xml_diff>
--- a/docs/Calendar.xlsx
+++ b/docs/Calendar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\fullstack\Personal Finance Management\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3687F7C-7FC2-4D34-A26C-00C8F5E4B7BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F67D13DE-81CE-450D-A3E8-8E4A722177DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
   <si>
     <t>BẢNG BIỂU KẾ HOẠCH</t>
   </si>
@@ -74,6 +74,9 @@
   </si>
   <si>
     <t>Hoàn thiện chức năng nâng cao: Liên kết đăng nhập (OAuth2), email xác thực (Java email seeder), ghi nhớ đăng nhập, revoke token (Redis), lưu ảnh hồ sơ (cloudinary)</t>
+  </si>
+  <si>
+    <t>Phát triển chức năng nâng cao: Liên kết tài khoản ngân hàng, tự động cập nhật thu chi</t>
   </si>
 </sst>
 </file>
@@ -120,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -140,7 +143,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -526,10 +528,12 @@
         <v>15</v>
       </c>
       <c r="E10" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F10" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
+      <c r="G10" s="6"/>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
     </row>
@@ -539,8 +543,8 @@
       <c r="C11" s="6"/>
       <c r="D11" s="6"/>
       <c r="E11" s="6"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
     </row>
@@ -550,8 +554,8 @@
       <c r="C12" s="6"/>
       <c r="D12" s="6"/>
       <c r="E12" s="6"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
       <c r="H12" s="3"/>
       <c r="I12" s="3"/>
     </row>
@@ -561,8 +565,8 @@
       <c r="C13" s="6"/>
       <c r="D13" s="6"/>
       <c r="E13" s="6"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
     </row>
@@ -572,8 +576,8 @@
       <c r="C14" s="6"/>
       <c r="D14" s="6"/>
       <c r="E14" s="6"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="6"/>
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
     </row>

</xml_diff>